<commit_message>
chore(corpus): re-emit 9 pre-reservoir-dropdown xlsx to clear cosmetic drift
gw015a/b, gw016a/b/c, gw021a/b (build_groundwater.py) and gs2_cons, gs2_infil
(benchmarks/geostudio) were built before the reservoir BC dropdown landed in
the template, so their embedded sharedStrings/dropdown list was one entry
short of the current template resource. Re-ran the owning builders to
regenerate all 9 from the current template.

Verified loader-level value-identity against the prior files (deep dict
compare via load_slope_data), confirmed the rebuild is content-reproducible
(unzipped xlsx contents match byte-for-byte across two independent builder
runs; only volatile zip/docProps timestamps differ), and reran run_tests.py
--tseep: 37/37 green, delta 0.000 on every tag, no lock moved.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0147GB4LGVZuqGHCRMVzZTsR
</commit_message>
<xml_diff>
--- a/docs/verification/files/geostudio/gs2_cons.xlsx
+++ b/docs/verification/files/geostudio/gs2_cons.xlsx
@@ -63,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="478" uniqueCount="265">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="480" uniqueCount="266">
   <si>
     <t>X</t>
   </si>
@@ -1023,6 +1023,9 @@
   </si>
   <si>
     <t>save_times</t>
+  </si>
+  <si>
+    <t>reservoir</t>
   </si>
 </sst>
 </file>
@@ -13837,7 +13840,9 @@
       <c r="O6" s="3"/>
       <c r="Q6" s="3"/>
       <c r="R6" s="3"/>
-      <c r="T6" s="1"/>
+      <c r="T6" s="1" t="s">
+        <v>265</v>
+      </c>
       <c r="U6" s="9"/>
     </row>
     <row r="7" spans="2:21" x14ac:dyDescent="0.2">
@@ -14103,7 +14108,7 @@
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E3 H3 K3 N3 Q3" xr:uid="{21F200C9-4829-4345-9958-0F754F272AD0}">
-      <formula1>$T$4:$T$5</formula1>
+      <formula1>$T$4:$T$6</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -14253,6 +14258,9 @@
       <c r="O6" s="3"/>
       <c r="Q6" s="3"/>
       <c r="R6" s="3"/>
+      <c r="T6" s="1" t="s">
+        <v>265</v>
+      </c>
     </row>
     <row r="7" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B7" s="3"/>
@@ -14517,7 +14525,7 @@
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E3 H3 K3 N3 Q3" xr:uid="{68C61D93-1721-F843-8E53-0F0E50006C65}">
-      <formula1>$T$4:$T$5</formula1>
+      <formula1>$T$4:$T$6</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>